<commit_message>
fix(templates): the analysis chart draws its axes where a column chart has them
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Co-authored-by: chiruotong <chiruotong@zhishi.local>
</commit_message>
<xml_diff>
--- a/backend/app/domain/documents/templates/analysis.xlsx
+++ b/backend/app/domain/documents/templates/analysis.xlsx
@@ -234,7 +234,8 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
-        <axPos val="l"/>
+        <delete val="0"/>
+        <axPos val="b"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="100"/>
@@ -245,8 +246,8 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
-        <majorGridlines/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="10"/>
@@ -270,7 +271,7 @@
       <row>1</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="5400000" cy="2700000"/>
+    <ext cx="5760000" cy="2880000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="1" name="Chart 1"/>

</xml_diff>